<commit_message>
WIP snapshot: Level 4 lessons still in review (not final)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVxwagJ2ocBAdfHuqZnXCC
</commit_message>
<xml_diff>
--- a/04-advanced-analysis/03-power-query/4.3-power-query.xlsx
+++ b/04-advanced-analysis/03-power-query/4.3-power-query.xlsx
@@ -265,14 +265,14 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:C32"/>
+  <dimension ref="B1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -696,6 +696,7 @@
     <col width="95" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -717,6 +718,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -773,6 +775,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
@@ -877,6 +880,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="B22" s="4" t="inlineStr">
         <is>
@@ -933,6 +937,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="B28" s="4" t="inlineStr">
         <is>
@@ -944,46 +949,82 @@
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Data Files</t>
+          <t>Practice</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Data: 6 rows</t>
+          <t>13 tasks. Build each query in Power Query, then type its result in the yellow cell.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="8" t="inlineStr">
         <is>
+          <t>Data Files</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>What each CSV file in the lesson's data folder contains. Power Query reads those files from disk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="33" customHeight="1">
+      <c r="B31" s="8" t="inlineStr">
+        <is>
           <t>DenialMap</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Data: 7 rows — Excel Table 'tblDenialMap'</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="63" customHeight="1">
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>About the data</t>
-        </is>
-      </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>CSV exports in the lesson's data folder: twelve monthly files of claims submitted in 2025, a January 2026 claim file (simulated next-month export) for the bonus, the payer list, 11,196 encounters discharged in 2025, and a wide 2025 budget-vs-actual export. The workbook adds a hand-maintained denial-reason mapping table.</t>
+          <t>Excel Table 'tblDenialMap': each denial reason and the team that works it. The Revenue Integrity team types it by hand (task 9).</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="8" t="inlineStr">
         <is>
+          <t>Starter M</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>The M code you paste into a blank query for task 11 (also in starter/AgedPending.m).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Bonus</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>A refreshable denial dashboard, then a January 2026 file and one click of Refresh All.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="63" customHeight="1">
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>About the data</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>CSV exports in the lesson's data folder: twelve monthly files of claims submitted in 2025, a January 2026 claim file (simulated next-month export) for the bonus, the payer list, 11,196 encounters discharged in 2025, and a wide 2025 budget-vs-actual export. The workbook adds a hand-maintained denial-reason mapping table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="B35" s="8" t="inlineStr">
+        <is>
           <t>Disclaimer</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>All people, places, and numbers are synthetic and fictional. Not clinical guidance.</t>
         </is>
@@ -1019,10 +1060,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="49" customHeight="1">
+    <row r="2" ht="64" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Build every query in this workbook from the CSV files in the lesson's data folder (Guide section 2), and do the tasks in order because later tasks reuse earlier queries. Type each result in the yellow cell as a plain number or text. From task 3 on, the answer key's M code uses a DataFolder parameter (Guide section 12). If you skip the parameter, or work on a Mac, your code shows your full folder path in its place.</t>
+          <t>Build every query in this workbook from the CSV files in the lesson's data folder (Guide section 2), and do the tasks in order because later tasks reuse earlier queries. Name each query as the task says, because later tasks and the answer key use those names. Type each result in the yellow cell as a plain number or text. From task 3 on, the answer key's M code uses a DataFolder parameter (Guide section 12). If you skip the parameter, or work on a Mac, your code shows your full folder path in its place.</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1137,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Import claims_2025_11.csv and claims_2025_12.csv as two more queries. Then, in the Power Query Editor, stack them with Home → Append Queries → Append Queries as New. How many rows does the appended query return?</t>
+          <t>Import claims_2025_11.csv and claims_2025_12.csv as two more queries. Then, in the Power Query Editor, stack them with Home → Append Queries → Append Queries as New, and name the new query Claims_NovDec. How many rows does it return?</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
@@ -1140,12 +1181,12 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>What is the total PaidAmount across all 2025 claims in your Claims query? Check that PaidAmount has the Decimal Number type (1.2 icon), then enter the total to the cent.</t>
+          <t>Check that PaidAmount in Claims has the Decimal Number type (1.2 icon). Then reference Claims in a new query named PaidTotal and total its PaidAmount column. What is the total PaidAmount across all 2025 claims? Enter it to the cent.</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>Reference Claims, then Transform → Statistics → Sum on PaidAmount</t>
+          <t>Select PaidAmount, then Transform → Statistics → Sum</t>
         </is>
       </c>
       <c r="D9" s="23" t="n"/>
@@ -1154,7 +1195,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="51" customHeight="1">
+    <row r="10" ht="66" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
           <t>5</t>
@@ -1162,7 +1203,7 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Reference Claims, keep only rows whose ClaimStatus is Denied, and use Home → Group By on DenialReason with the operation Count Rows. How many denied claims list Authorization Required as the reason?</t>
+          <t>Reference Claims in a new query named DenialsByReason, keep only rows whose ClaimStatus is Denied, and use Home → Group By on DenialReason with the operation Count Rows. How many denied claims list Authorization Required as the reason?</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
@@ -1206,7 +1247,7 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Import payers.csv as a query named Payers. Then reference Claims, merge it with Payers on PayerID (Join Kind: Left Outer), expand only PayerType, and group by PayerType with Sum of PaidAmount. What was the total PaidAmount for the Commercial payer type? Enter it to the cent.</t>
+          <t>Import payers.csv as a query named Payers. Then reference Claims in a new query named PaidByPayerType, merge it with Payers on PayerID (Join Kind: Left Outer), expand only PayerType, and group by PayerType with Sum of PaidAmount. What was the total PaidAmount for the Commercial payer type? Enter it to the cent.</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
@@ -1228,12 +1269,12 @@
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>Reference Claims and add a custom column DaysToSubmit that holds the number of days from ServiceDate to SubmitDate. How many 2025 claims took MORE than 30 days to submit?</t>
+          <t>Reference Claims in a new query named SubmitLag and add a custom column DaysToSubmit that holds the number of days from ServiceDate to SubmitDate, with the Whole Number type. How many 2025 claims took MORE than 30 days to submit?</t>
         </is>
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
-          <t>Add Column → Custom Column, then Duration.Days of the date difference</t>
+          <t>Duration.Days turns a date difference into days. Then Number Filters → Greater Than, and count the rows</t>
         </is>
       </c>
       <c r="D13" s="21" t="n"/>
@@ -1250,7 +1291,7 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Load tblDenialMap (on the DenialMap sheet) with Data → From Table/Range and name the query DenialMap. Reference Claims, keep the Denied rows, merge them with the map on DenialReason (Left Outer), and expand OwnerTeam. Check that EVERY denied claim found a match (no null OwnerTeam), and fix the keys in the map query if some didn't. What is the total denied BilledAmount owned by Patient Access? Enter it to the cent.</t>
+          <t>Load tblDenialMap (on the DenialMap sheet) with Data → From Table/Range and name the query DenialMap. Reference Claims in a new query named DenialsByOwner, keep the Denied rows, merge them with the map on DenialReason (Left Outer), and expand OwnerTeam. Check that EVERY denied claim found a match (no null OwnerTeam), and fix the keys in the map query if some didn't. What is the total denied BilledAmount owned by Patient Access? Enter it to the cent.</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
@@ -1272,7 +1313,7 @@
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>Import encounters_2025.csv (one row per encounter discharged in 2025) as a query named Encounters2025. Use Merge Queries as New with Encounters2025 on top, Claims below, EncounterID in both, and Join Kind Left Anti. How many 2025 encounters have no claim in the 2025 claim files?</t>
+          <t>Import encounters_2025.csv (one row per encounter discharged in 2025) as a query named Encounters2025. Use Merge Queries as New with Encounters2025 on top, Claims below, EncounterID in both, and Join Kind Left Anti. Name the new query Unbilled. How many 2025 encounters have no claim in the 2025 claim files?</t>
         </is>
       </c>
       <c r="C15" s="20" t="inlineStr">
@@ -1330,7 +1371,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="81" customHeight="1">
+    <row r="18" ht="96" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
         <is>
           <t>13</t>
@@ -1338,12 +1379,12 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>In Budget2025, split Department (for example '6130 - Intensive Care Unit') into CostCenter and DeptName with Transform → Split Column → By Delimiter, using ' - ' (space, hyphen, space) at the left-most delimiter. What was the Q1 2025 (Jan–Mar) Actual Salaries &amp; Wages for all three departments named Intensive Care Unit combined? Enter whole dollars.</t>
+          <t>In Budget2025, split Department (for example '6130 - Intensive Care Unit') into CostCenter and DeptName with Transform → Split Column → By Delimiter, using ' - ' (space, hyphen, space) at the left-most delimiter. Then reference Budget2025 in a new query named ICU_Q1_Salaries. What was the Q1 2025 (Jan–Mar) Actual Salaries &amp; Wages for all three departments named Intensive Care Unit combined? Enter whole dollars.</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>Filter DeptName, Category, Measure, and Month, then Group By or Sum</t>
+          <t>Filter DeptName, Category, Measure, and Month, then Transform → Statistics → Sum on Amount (or Group By)</t>
         </is>
       </c>
       <c r="D18" s="21" t="n"/>
@@ -1517,20 +1558,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="25" t="inlineStr">
         <is>
-          <t>Denial reason → owner team (maintained by hand by the Revenue Integrity team)</t>
+          <t>Denial reason → owner team (typed by hand)</t>
         </is>
       </c>
     </row>
@@ -1544,7 +1585,7 @@
     <row r="3">
       <c r="A3" s="26" t="inlineStr">
         <is>
-          <t>Each denial reason should appear once. OwnerTeam is the department that fixes that kind of denial.</t>
+          <t>Each reason should appear once. OwnerTeam is the team that works that kind of denial.</t>
         </is>
       </c>
     </row>
@@ -1686,6 +1727,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -1697,7 +1739,7 @@
   <sheetPr>
     <tabColor rgb="007030A0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1712,99 +1754,106 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="31" t="inlineStr">
-        <is>
-          <t>Select A4:A16, copy (Ctrl + C, Mac: ⌘ + C), then paste into Home → Advanced Editor of a new Blank Query, replacing everything there. The same code is in starter/AgedPending.m.</t>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Select A4:A16, copy (Ctrl + C, Mac: ⌘ + C), then paste into Home → Advanced Editor of a new Blank Query.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Replace everything that was in the Advanced Editor window. The same code is in starter/AgedPending.m.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="32" t="inlineStr">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>// AgedPending: Pending claims that have waited too long for payment.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="32" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>// Paste into Data &gt; Get Data &gt; From Other Sources &gt; Blank Query &gt; Home &gt; Advanced Editor.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="32" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>// It reads your Claims query (task 3), so that query must exist and be named Claims.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="32" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>let</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="32" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">    Source = Claims,</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">    AsOf = #date(2025, 12, 31),</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">    PendingOnly = Table.SelectRows(Source, each [ClaimStatus] = "Pending"),</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="32" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">    AddDaysPending = Table.AddColumn(PendingOnly, "DaysPending", each Duration.Days(AsOf - [SubmitDate]), Int64.Type),</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">    Aged = Table.SelectRows(AddDaysPending, each [DaysPending] &gt; 60),</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="32" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">    KeepColumns = Table.SelectColumns(Aged, {"ClaimID", "PayerID", "SubmitDate", "BilledAmount", "DaysPending"}),</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">    Sorted = Table.Sort(KeepColumns, {{"DaysPending", Order.Descending}})</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="32" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>in</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="32" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">    Sorted</t>
         </is>
@@ -1812,6 +1861,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1899,7 +1949,7 @@
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>Ctrl-click two columns in the Group By dialog (Advanced)</t>
+          <t>Select PayerType and DenialReason before you click Group By, or use Add grouping in the Advanced dialog</t>
         </is>
       </c>
       <c r="D6" s="23" t="n"/>
@@ -1908,7 +1958,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="66" customHeight="1">
+    <row r="7" ht="81" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
           <t>B2</t>
@@ -1916,12 +1966,12 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Build DenialRateByPayerType from ALL claims: reference Claims, merge Payers for PayerType, add a conditional column IsDenied (1 if ClaimStatus is Denied, otherwise 0), then group by PayerType with Count Rows and Sum of IsDenied. Which payer type has the highest denial rate (denied claims ÷ all claims)?</t>
+          <t>Build a query named DenialRateByPayerType from ALL claims: reference Claims, merge Payers for PayerType, and add a conditional column IsDenied (1 if ClaimStatus is Denied, otherwise 0). Group by PayerType with two aggregations: AllClaims (Count Rows) and Denied (Sum of IsDenied). Which payer type has the highest denial rate (denied claims ÷ all claims)?</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>Add Column → Conditional Column, then a custom column Denied / AllClaims</t>
+          <t>After the Group By step, add a custom column DenialRate = [Denied] / [AllClaims] and sort it</t>
         </is>
       </c>
       <c r="D7" s="24" t="n"/>
@@ -1943,10 +1993,10 @@
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>Format the DenialRate column as Percentage</t>
-        </is>
-      </c>
-      <c r="D8" s="33" t="n"/>
+          <t>Click the type icon in the DenialRate header and choose Percentage</t>
+        </is>
+      </c>
+      <c r="D8" s="32" t="n"/>
       <c r="E8" s="22">
         <f>IF(IFERROR(D8="",FALSE),"",IF(IFERROR(AND(ISNUMBER(D8),OR(ABS(D8-'Bonus Key'!$C$7)&lt;=0.00051,ABS(D8-'Bonus Key'!$C$7*100)&lt;=0.051000000000000004)),FALSE),"✔ Correct","✘ Not yet"))</f>
         <v/>
@@ -2028,22 +2078,22 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="34" t="inlineStr">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>🔑 Answer Key — Lesson 4.3</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="31" t="inlineStr">
-        <is>
-          <t>Spoiler alert — try every task before reading this sheet. Column C is the value the Check column compares against. Column D is a sample solution; column E is that same formula, live, proving it works.</t>
+    <row r="2" ht="47" customHeight="1">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>Spoiler alert: try every task before reading this sheet. Column C is the value the Check column compares against. Column D is the M code (or the steps) that produces it. Long code is cut off in its cell, so click the cell and read it in the formula bar, or open the matching .m file in the lesson's solutions folder. Column E is blank because Power Query results can't be recalculated by a cell formula.</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2129,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="336" customHeight="1">
+    <row r="5" ht="175" customHeight="1">
       <c r="A5" s="18" t="inlineStr">
         <is>
           <t>1</t>
@@ -2116,7 +2166,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="171" customHeight="1">
+    <row r="6" ht="110" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>2</t>
@@ -2124,7 +2174,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Import claims_2025_11.csv and claims_2025_12.csv as two more queries. Then, in the Power Query Editor, stack them with Home → Append Queries → Append Queries as New. How many rows does the appended query return?</t>
+          <t>Import claims_2025_11.csv and claims_2025_12.csv as two more queries. Then, in the Power Query Editor, stack them with Home → Append Queries → Append Queries as New, and name the new query Claims_NovDec. How many rows does it return?</t>
         </is>
       </c>
       <c r="C6" s="36" t="n">
@@ -2202,7 +2252,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="216" customHeight="1">
+    <row r="8" ht="136" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
           <t>4</t>
@@ -2210,7 +2260,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>What is the total PaidAmount across all 2025 claims in your Claims query? Check that PaidAmount has the Decimal Number type (1.2 icon), then enter the total to the cent.</t>
+          <t>Check that PaidAmount in Claims has the Decimal Number type (1.2 icon). Then reference Claims in a new query named PaidTotal and total its PaidAmount column. What is the total PaidAmount across all 2025 claims? Enter it to the cent.</t>
         </is>
       </c>
       <c r="C8" s="38" t="n">
@@ -2239,7 +2289,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="201" customHeight="1">
+    <row r="9" ht="123" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
           <t>5</t>
@@ -2247,7 +2297,7 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Reference Claims, keep only rows whose ClaimStatus is Denied, and use Home → Group By on DenialReason with the operation Count Rows. How many denied claims list Authorization Required as the reason?</t>
+          <t>Reference Claims in a new query named DenialsByReason, keep only rows whose ClaimStatus is Denied, and use Home → Group By on DenialReason with the operation Count Rows. How many denied claims list Authorization Required as the reason?</t>
         </is>
       </c>
       <c r="C9" s="36" t="n">
@@ -2276,7 +2326,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="291" customHeight="1">
+    <row r="10" ht="162" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
           <t>6</t>
@@ -2318,7 +2368,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="409" customHeight="1">
+    <row r="11" ht="305" customHeight="1">
       <c r="A11" s="18" t="inlineStr">
         <is>
           <t>7</t>
@@ -2326,7 +2376,7 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>Import payers.csv as a query named Payers. Then reference Claims, merge it with Payers on PayerID (Join Kind: Left Outer), expand only PayerType, and group by PayerType with Sum of PaidAmount. What was the total PaidAmount for the Commercial payer type? Enter it to the cent.</t>
+          <t>Import payers.csv as a query named Payers. Then reference Claims in a new query named PaidByPayerType, merge it with Payers on PayerID (Join Kind: Left Outer), expand only PayerType, and group by PayerType with Sum of PaidAmount. What was the total PaidAmount for the Commercial payer type? Enter it to the cent.</t>
         </is>
       </c>
       <c r="C11" s="38" t="n">
@@ -2364,7 +2414,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="171" customHeight="1">
+    <row r="12" ht="111" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
           <t>8</t>
@@ -2372,7 +2422,7 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Reference Claims and add a custom column DaysToSubmit that holds the number of days from ServiceDate to SubmitDate. How many 2025 claims took MORE than 30 days to submit?</t>
+          <t>Reference Claims in a new query named SubmitLag and add a custom column DaysToSubmit that holds the number of days from ServiceDate to SubmitDate, with the Whole Number type. How many 2025 claims took MORE than 30 days to submit?</t>
         </is>
       </c>
       <c r="C12" s="36" t="n">
@@ -2400,7 +2450,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="409" customHeight="1">
+    <row r="13" ht="331" customHeight="1">
       <c r="A13" s="18" t="inlineStr">
         <is>
           <t>9</t>
@@ -2408,7 +2458,7 @@
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>Load tblDenialMap (on the DenialMap sheet) with Data → From Table/Range and name the query DenialMap. Reference Claims, keep the Denied rows, merge them with the map on DenialReason (Left Outer), and expand OwnerTeam. Check that EVERY denied claim found a match (no null OwnerTeam), and fix the keys in the map query if some didn't. What is the total denied BilledAmount owned by Patient Access? Enter it to the cent.</t>
+          <t>Load tblDenialMap (on the DenialMap sheet) with Data → From Table/Range and name the query DenialMap. Reference Claims in a new query named DenialsByOwner, keep the Denied rows, merge them with the map on DenialReason (Left Outer), and expand OwnerTeam. Check that EVERY denied claim found a match (no null OwnerTeam), and fix the keys in the map query if some didn't. What is the total denied BilledAmount owned by Patient Access? Enter it to the cent.</t>
         </is>
       </c>
       <c r="C13" s="38" t="n">
@@ -2448,7 +2498,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="409" customHeight="1">
+    <row r="14" ht="292" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
         <is>
           <t>10</t>
@@ -2456,7 +2506,7 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Import encounters_2025.csv (one row per encounter discharged in 2025) as a query named Encounters2025. Use Merge Queries as New with Encounters2025 on top, Claims below, EncounterID in both, and Join Kind Left Anti. How many 2025 encounters have no claim in the 2025 claim files?</t>
+          <t>Import encounters_2025.csv (one row per encounter discharged in 2025) as a query named Encounters2025. Use Merge Queries as New with Encounters2025 on top, Claims below, EncounterID in both, and Join Kind Left Anti. Name the new query Unbilled. How many 2025 encounters have no claim in the 2025 claim files?</t>
         </is>
       </c>
       <c r="C14" s="36" t="n">
@@ -2487,11 +2537,11 @@
       </c>
       <c r="F14" s="19" t="inlineStr">
         <is>
-          <t>A Left Anti join keeps only the rows in the first table that have no match in the second. It's the fastest way to answer "what's missing?" questions. These encounters were discharged but not yet billed (hospitals call this *discharged not final billed*, or DNFB), and together they carry $2,371,213.36 of charges. Name the query Unbilled, because the bonus refreshes it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="351" customHeight="1">
+          <t>A Left Anti join keeps only the rows in the first table that have no match in the second. It's the fastest way to answer "what's missing?" questions. These encounters were discharged but not yet billed (hospitals call this *discharged not final billed*, or DNFB), and together they carry $2,371,213.36 of charges. The bonus refreshes this list after the January 2026 claims arrive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="201" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
         <is>
           <t>11</t>
@@ -2533,7 +2583,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="409" customHeight="1">
+    <row r="16" ht="279" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
           <t>12</t>
@@ -2582,7 +2632,7 @@
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>In Budget2025, split Department (for example '6130 - Intensive Care Unit') into CostCenter and DeptName with Transform → Split Column → By Delimiter, using ' - ' (space, hyphen, space) at the left-most delimiter. What was the Q1 2025 (Jan–Mar) Actual Salaries &amp; Wages for all three departments named Intensive Care Unit combined? Enter whole dollars.</t>
+          <t>In Budget2025, split Department (for example '6130 - Intensive Care Unit') into CostCenter and DeptName with Transform → Split Column → By Delimiter, using ' - ' (space, hyphen, space) at the left-most delimiter. Then reference Budget2025 in a new query named ICU_Q1_Salaries. What was the Q1 2025 (Jan–Mar) Actual Salaries &amp; Wages for all three departments named Intensive Care Unit combined? Enter whole dollars.</t>
         </is>
       </c>
       <c r="C17" s="36" t="n">
@@ -2648,22 +2698,22 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="34" t="inlineStr">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>🔑 Bonus Key — Lesson 4.3</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="31" t="inlineStr">
-        <is>
-          <t>Spoiler alert — try every task before reading this sheet. Column C is the value the Check column compares against. Column D is a sample solution; column E is that same formula, live, proving it works.</t>
+    <row r="2" ht="47" customHeight="1">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>Spoiler alert: try every task before reading this sheet. Column C is the value the Check column compares against. Column D is the M code (or the steps) that produces it. Long code is cut off in its cell, so click the cell and read it in the formula bar, or open the matching .m file in the lesson's solutions folder. Column E is blank because Power Query results can't be recalculated by a cell formula.</t>
         </is>
       </c>
     </row>
@@ -2699,7 +2749,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="336" customHeight="1">
+    <row r="5" ht="188" customHeight="1">
       <c r="A5" s="18" t="inlineStr">
         <is>
           <t>B1</t>
@@ -2740,7 +2790,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="409" customHeight="1">
+    <row r="6" ht="227" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>B2</t>
@@ -2748,7 +2798,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Build DenialRateByPayerType from ALL claims: reference Claims, merge Payers for PayerType, add a conditional column IsDenied (1 if ClaimStatus is Denied, otherwise 0), then group by PayerType with Count Rows and Sum of IsDenied. Which payer type has the highest denial rate (denied claims ÷ all claims)?</t>
+          <t>Build a query named DenialRateByPayerType from ALL claims: reference Claims, merge Payers for PayerType, and add a conditional column IsDenied (1 if ClaimStatus is Denied, otherwise 0). Group by PayerType with two aggregations: AllClaims (Count Rows) and Denied (Sum of IsDenied). Which payer type has the highest denial rate (denied claims ÷ all claims)?</t>
         </is>
       </c>
       <c r="C6" s="36" t="inlineStr">
@@ -2784,7 +2834,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="66" customHeight="1">
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
           <t>B3</t>

</xml_diff>